<commit_message>
fix: update Mirth Connect Channel and XSLT files to correct the grouper observation resource ID generation logic #3124 - Updated the Grouper Observation Resource ID generation logic to select the first valid OBR with a non-empty OBR.26 value and at least one valid child OBX containing an allowed screening question code and a non-empty/non-UNK observation value. Removed the checking of specific screening codes ("96777-8", "97023-6", "NYSAHCHRSN", "NYS-AHC-HRSN"). - Updated HL7 to FHIR conversion specification document.
</commit_message>
<xml_diff>
--- a/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
+++ b/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="753" firstSheet="1" activeTab="5"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="753" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="469">
   <si>
     <t>FHIR Resources</t>
   </si>
@@ -350,6 +350,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Uses the </t>
     </r>
     <r>
@@ -486,6 +492,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Uses the </t>
     </r>
     <r>
@@ -3514,7 +3526,7 @@
     <t>SHA-256 UUID generated using 
 1. Patient MRN (PID.3.1)
 2. Patient CIN from the header variable 'X-TechBD-CIN'
-3. Organization Name from the header variable 'X-TechBD-Organization-Name'
+3. Organization Name from the header variable 'X-TechBD-Organization-Name' OR MSH.6
 4. Organization NPI from the header variable 'X-TechBD-OrgNPI'
 5. Organization TIN from the header variable 'X-TechBD-OrgTIN'
 6. Organization Address (ORC.22)
@@ -3826,7 +3838,7 @@
     <t>name</t>
   </si>
   <si>
-    <t>X-TechBD-Organization-Name</t>
+    <t>X-TechBD-Organization-Name OR MSH.6</t>
   </si>
   <si>
     <t>"name" : "Care Ridge SCN",</t>
@@ -3840,18 +3852,39 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Mapped from the header variable,  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>X-TechBD-Organization-Name</t>
+      <t xml:space="preserve">If the header variable,  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">X-TechBD-Organization-Name </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">is not set, it will take from </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MSH.6</t>
     </r>
   </si>
   <si>
@@ -4314,14 +4347,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Question Code -&gt; Category Display Mapping</t>
     </r>
     <r>
@@ -4551,6 +4576,66 @@
           } ]</t>
   </si>
   <si>
+    <t>interpretation  -&gt; coding -&gt; system</t>
+  </si>
+  <si>
+    <t>"http://terminology.hl7.org/CodeSystem/v3-ObservationInterpretation"</t>
+  </si>
+  <si>
+    <t>"interpretation": [
+          {
+            "coding": [
+              {
+                "system": "http://terminology.hl7.org/CodeSystem/v3-ObservationInterpretation",
+                "code": "L",
+                "display": "Low"
+              }
+            ]
+          }
+        ],</t>
+  </si>
+  <si>
+    <t>interpretation  -&gt; coding -&gt; code</t>
+  </si>
+  <si>
+    <t>OBX.8</t>
+  </si>
+  <si>
+    <t>interpretation  -&gt; coding -&gt; display</t>
+  </si>
+  <si>
+    <r>
+      <t>Interpretation Code -&gt; Interpretation Display Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+L -&gt; Low
+H -&gt; High
+LL -&gt; Critical low
+HH -&gt; Critical high
+N -&gt; Normal
+A -&gt; Abnormal
+AA -&gt; Critical abnormal
+U -&gt; Significant change up
+D -&gt; Significant change down
+B -&gt; Better
+W -&gt; Worse
+S -&gt; Susceptible
+R -&gt; Resistant
+I -&gt; Intermediate
+MS -&gt; Moderately susceptible
+VS -&gt; Very susceptible
+CAR -&gt; Carrier</t>
+    </r>
+  </si>
+  <si>
     <t>issued</t>
   </si>
   <si>
@@ -4796,7 +4881,8 @@
 SHA-256 UUID generated using 
 1. Patient MRN (PID.3.1)
 2. Patient CIN from the header variable 'X-TechBD-CIN'
-3. Content of the first OBX segment where the code is one of ("96777-8", "97023-6", "NYSAHCHRSN", "NYS-AHC-HRSN")</t>
+3. SHA-256 UUID generated using the content of first OBX segment
+4. Content of the first valid OBR segment with a non-empty OBR.26 value and at least one valid child OBX containing an allowed screening question code and a non-empty/non-UNK observation value.</t>
   </si>
   <si>
     <t>"id" : "ACPNY-96777-8cae0e5315917a2fd2a53faf4ebe45e26f5bc6b79eeec",</t>
@@ -4888,7 +4974,7 @@
     <t>It will list the categories present in all the observations. Also item for "social-history" and "Survey".</t>
   </si>
   <si>
-    <t>OBR.26</t>
+    <t>First part of OBR.26 (split by '&amp;')</t>
   </si>
   <si>
     <r>
@@ -5302,12 +5388,21 @@
       },</t>
   </si>
   <si>
+    <t>OBX.14.1/OBR.7.1/OBR.8.1/meta.lastUpdated</t>
+  </si>
+  <si>
+    <t>If OBX.14.1/OBR.7.1/OBR.8.1 is not valued, then use the same timestamp that is used in the meta.lastUpdated.</t>
+  </si>
+  <si>
     <t>performer</t>
   </si>
   <si>
     <t>"performer": [ {
             "reference": "Organization/UMC20250121T1024400530"
           } ]</t>
+  </si>
+  <si>
+    <t>From the first valid OBX with non-empty OBX.8 under the selected OBR.</t>
   </si>
   <si>
     <t>Path to get the issued date time</t>
@@ -5408,6 +5503,15 @@
       <b/>
       <u/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5499,15 +5603,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF333333"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5726,9 +5821,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF00B050"/>
+      <b/>
+      <sz val="11"/>
+      <color indexed="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -5743,13 +5844,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -5758,22 +5852,23 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="10"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="40">
@@ -6301,7 +6396,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6348,45 +6443,45 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
@@ -6395,40 +6490,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -6437,43 +6529,40 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6591,7 +6680,7 @@
     <cellStyle name="Warning" xfId="59"/>
   </cellStyles>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{3D1CA4B2-FB8F-44D4-890D-8FC6844F2DFA}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{58ECC587-4D15-4AA1-90CF-3197D7A288C3}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -6862,66 +6951,66 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="11.8571428571429" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="14.2857142857143" style="72" customWidth="1"/>
+    <col min="1" max="1" width="14.2857142857143" style="70" customWidth="1"/>
     <col min="2" max="2" width="47" customWidth="1"/>
     <col min="3" max="3" width="123.571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67" t="s">
+      <c r="A2" s="65"/>
+      <c r="B2" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="59" t="s">
+      <c r="C2" s="57" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="67"/>
-      <c r="B3" s="67" t="s">
+      <c r="A3" s="65"/>
+      <c r="B3" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="C3" s="57" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="67"/>
-      <c r="B4" s="67" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="59" t="s">
+      <c r="C4" s="57" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="45" spans="1:3">
-      <c r="A5" s="67"/>
-      <c r="B5" s="67" t="s">
+      <c r="A5" s="65"/>
+      <c r="B5" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="69" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="67"/>
-      <c r="B6" s="71" t="s">
+      <c r="A6" s="65"/>
+      <c r="B6" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="59" t="s">
+      <c r="C6" s="57" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="67"/>
-      <c r="B7" s="67" t="s">
+      <c r="A7" s="65"/>
+      <c r="B7" s="65" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="13" t="s">
@@ -6929,8 +7018,8 @@
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="67"/>
-      <c r="B8" s="67" t="s">
+      <c r="A8" s="65"/>
+      <c r="B8" s="65" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="13" t="s">
@@ -6947,7 +7036,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="14.7142857142857" style="2" customWidth="1"/>
@@ -6967,16 +7056,16 @@
         <v>16</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
     </row>
     <row r="2" s="2" customFormat="1" ht="17" customHeight="1" spans="1:6">
@@ -6998,16 +7087,16 @@
         <v>343</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" ht="135" spans="1:6">
+    <row r="4" s="2" customFormat="1" ht="180" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" spans="1:6">
@@ -7027,7 +7116,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -7042,10 +7131,10 @@
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="74.25" spans="1:6">
@@ -7053,13 +7142,13 @@
         <v>189</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>349</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="409" customHeight="1" spans="1:6">
@@ -7068,10 +7157,10 @@
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="5" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="150" spans="1:6">
@@ -7079,13 +7168,13 @@
         <v>360</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="180" spans="1:6">
@@ -7095,7 +7184,7 @@
       <c r="C11" s="5"/>
       <c r="D11" s="2"/>
       <c r="E11" s="12" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="150" spans="1:6">
@@ -7105,7 +7194,7 @@
       <c r="C12" s="5"/>
       <c r="D12" s="2"/>
       <c r="E12" s="12" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="75" spans="1:6">
@@ -7116,7 +7205,7 @@
         <v>382</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="30" spans="1:6">
@@ -7135,7 +7224,7 @@
         <v>385</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="30" spans="1:6">
@@ -7143,74 +7232,108 @@
         <v>387</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>411</v>
+        <v>459</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>389</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>390</v>
+        <v>460</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="45" spans="2:6">
       <c r="B17" s="6" t="s">
-        <v>452</v>
+        <v>461</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>221</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="18" s="2" customFormat="1" spans="2:6">
-      <c r="B18" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="18" s="2" customFormat="1" ht="30" spans="2:6">
+      <c r="B18" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2" t="s">
+      <c r="C18" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="15" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="19" s="2" customFormat="1" ht="165" spans="2:6">
-      <c r="B19" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>456</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="20" s="2" customFormat="1" spans="2:6">
-      <c r="B20" s="5" t="s">
+    </row>
+    <row r="19" s="2" customFormat="1" ht="30" spans="2:6">
+      <c r="B19" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="20" s="2" customFormat="1" ht="270" spans="2:6">
+      <c r="B20" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="15" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="21" s="2" customFormat="1" spans="2:6">
+      <c r="B21" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="16" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="22" s="2" customFormat="1" ht="165" spans="2:6">
+      <c r="B22" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="23" s="2" customFormat="1" spans="2:6">
+      <c r="B23" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D20" s="16" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="21" s="2" customFormat="1" ht="46" customHeight="1" spans="2:6">
-      <c r="B21" s="5" t="s">
+      <c r="D23" s="17" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="24" s="2" customFormat="1" ht="46" customHeight="1" spans="2:6">
+      <c r="B24" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="C24" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="D24" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="D23:D24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -7223,24 +7346,24 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" style="67" customWidth="1"/>
-    <col min="2" max="2" width="28.2857142857143" style="67" customWidth="1"/>
-    <col min="3" max="3" width="62.7238095238095" style="67" customWidth="1"/>
-    <col min="4" max="4" width="54.5428571428571" style="67" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" style="65" customWidth="1"/>
+    <col min="2" max="2" width="28.2857142857143" style="65" customWidth="1"/>
+    <col min="3" max="3" width="62.7238095238095" style="65" customWidth="1"/>
+    <col min="4" max="4" width="54.5428571428571" style="65" customWidth="1"/>
     <col min="5" max="5" width="57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="68" t="s">
+      <c r="D1" s="66" t="s">
         <v>18</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -7248,32 +7371,32 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="67" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="69"/>
-      <c r="B3" s="67" t="s">
+      <c r="A3" s="67"/>
+      <c r="B3" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="65" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="69"/>
-      <c r="B4" s="67" t="s">
+      <c r="A4" s="67"/>
+      <c r="B4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="67" t="s">
+      <c r="D4" s="65" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" s="66" customFormat="1" ht="61" customHeight="1" spans="1:5">
+    <row r="5" s="64" customFormat="1" ht="61" customHeight="1" spans="1:5">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>26</v>
@@ -7285,7 +7408,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" s="66" customFormat="1" ht="49" customHeight="1" spans="1:5">
+    <row r="6" s="64" customFormat="1" ht="49" customHeight="1" spans="1:5">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>29</v>
@@ -7295,7 +7418,7 @@
       </c>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" s="66" customFormat="1" ht="316" customHeight="1" spans="1:5">
+    <row r="7" s="64" customFormat="1" ht="316" customHeight="1" spans="1:5">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>31</v>
@@ -7306,27 +7429,27 @@
       <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="67" t="s">
+      <c r="C8" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="71"/>
+      <c r="D8" s="69"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="67" t="s">
+      <c r="C9" s="65" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" ht="30" spans="1:5">
-      <c r="B10" s="67" t="s">
+      <c r="B10" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="71" t="s">
+      <c r="C10" s="69" t="s">
         <v>38</v>
       </c>
     </row>
@@ -7366,11 +7489,11 @@
       <c r="C17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="49" t="s">
+      <c r="E17" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
     </row>
     <row r="18" s="2" customFormat="1" ht="30" spans="1:7">
       <c r="B18" s="5" t="s">
@@ -7408,10 +7531,10 @@
       <c r="C22"/>
     </row>
     <row r="23" hidden="1" spans="1:7">
-      <c r="B23" s="67" t="s">
+      <c r="B23" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="71" t="s">
+      <c r="C23" s="69" t="s">
         <v>48</v>
       </c>
     </row>
@@ -7441,69 +7564,69 @@
     <col min="6" max="256" width="11.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="19" customFormat="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+    <row r="1" s="20" customFormat="1" spans="1:5">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="25"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="19"/>
+      <c r="A3" s="20"/>
       <c r="B3" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="26"/>
     </row>
     <row r="4" ht="60" spans="1:5">
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="48" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="20"/>
+      <c r="B5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="25"/>
+      <c r="E5" s="26"/>
     </row>
     <row r="6" ht="30" spans="1:5">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="25"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" ht="60" spans="1:5">
       <c r="B7" s="14" t="s">
@@ -7515,7 +7638,7 @@
       <c r="D7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="48" t="s">
         <v>57</v>
       </c>
     </row>
@@ -7529,16 +7652,16 @@
       <c r="D8" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="25"/>
+      <c r="E8" s="26"/>
     </row>
     <row r="9" spans="1:5">
       <c r="B9" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="59" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="25"/>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5">
       <c r="B10" s="14" t="s">
@@ -7550,10 +7673,10 @@
       <c r="D10" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="25"/>
+      <c r="E10" s="26"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="22" t="s">
         <v>66</v>
       </c>
       <c r="C11" s="14" t="s">
@@ -7562,10 +7685,10 @@
       <c r="D11" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="25"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="22" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -7574,7 +7697,7 @@
       <c r="D12" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="25"/>
+      <c r="E12" s="26"/>
     </row>
     <row r="13" ht="60" spans="1:5">
       <c r="B13" s="14" t="s">
@@ -7586,7 +7709,7 @@
       <c r="D13" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E13" s="25"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" ht="30" spans="1:5">
       <c r="B14" s="14" t="s">
@@ -7598,10 +7721,10 @@
       <c r="D14" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="22" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -7610,10 +7733,10 @@
       <c r="D15" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="22" t="s">
         <v>80</v>
       </c>
       <c r="C16" s="14" t="s">
@@ -7622,7 +7745,7 @@
       <c r="D16" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" ht="135" spans="2:5">
       <c r="B17" s="14" t="s">
@@ -7634,7 +7757,7 @@
       <c r="D17" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="E17" s="25"/>
+      <c r="E17" s="26"/>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="14" t="s">
@@ -7643,7 +7766,7 @@
       <c r="C18" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="E18" s="25"/>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="14" t="s">
@@ -7652,7 +7775,7 @@
       <c r="C19" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="25"/>
+      <c r="E19" s="26"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="14" t="s">
@@ -7661,7 +7784,7 @@
       <c r="C20" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="25"/>
+      <c r="E20" s="26"/>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="14" t="s">
@@ -7670,7 +7793,7 @@
       <c r="C21" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="E21" s="25"/>
+      <c r="E21" s="26"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="14" t="s">
@@ -7679,7 +7802,7 @@
       <c r="C22" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="E22" s="25"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" ht="90" spans="2:5">
       <c r="B23" s="14" t="s">
@@ -7702,7 +7825,7 @@
       <c r="D24" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="E24" s="49" t="s">
+      <c r="E24" s="48" t="s">
         <v>102</v>
       </c>
     </row>
@@ -7713,16 +7836,16 @@
       <c r="C25" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="E25" s="25"/>
+      <c r="E25" s="26"/>
     </row>
     <row r="26" ht="30" spans="2:5">
       <c r="B26" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="E26" s="51"/>
+      <c r="E26" s="15"/>
     </row>
     <row r="27" ht="45" spans="2:5">
       <c r="B27" s="30" t="s">
@@ -7731,7 +7854,7 @@
       <c r="C27" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="62" t="s">
+      <c r="D27" s="60" t="s">
         <v>109</v>
       </c>
       <c r="E27" s="9" t="s">
@@ -7745,8 +7868,8 @@
       <c r="C28" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="D28" s="62"/>
-      <c r="E28" s="63"/>
+      <c r="D28" s="60"/>
+      <c r="E28" s="61"/>
     </row>
     <row r="29" ht="30" spans="2:5">
       <c r="B29" s="30" t="s">
@@ -7755,8 +7878,8 @@
       <c r="C29" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="61"/>
     </row>
     <row r="30" ht="30" spans="2:5">
       <c r="B30" s="30" t="s">
@@ -7765,8 +7888,8 @@
       <c r="C30" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="D30" s="62"/>
-      <c r="E30" s="63"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="61"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="30" t="s">
@@ -7775,7 +7898,7 @@
       <c r="C31" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D31" s="62"/>
+      <c r="D31" s="60"/>
       <c r="E31" s="9"/>
     </row>
     <row r="32" ht="30" spans="2:5">
@@ -7785,7 +7908,7 @@
       <c r="C32" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D32" s="62" t="s">
+      <c r="D32" s="60" t="s">
         <v>119</v>
       </c>
       <c r="E32" s="9" t="s">
@@ -7799,8 +7922,8 @@
       <c r="C33" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="D33" s="62"/>
-      <c r="E33" s="63"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="61"/>
     </row>
     <row r="34" ht="30" spans="2:5">
       <c r="B34" s="30" t="s">
@@ -7809,8 +7932,8 @@
       <c r="C34" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="D34" s="62"/>
-      <c r="E34" s="63"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="61"/>
     </row>
     <row r="35" ht="30" spans="2:5">
       <c r="B35" s="30" t="s">
@@ -7819,8 +7942,8 @@
       <c r="C35" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="D35" s="62"/>
-      <c r="E35" s="63"/>
+      <c r="D35" s="60"/>
+      <c r="E35" s="61"/>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="30" t="s">
@@ -7829,8 +7952,8 @@
       <c r="C36" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D36" s="62"/>
-      <c r="E36" s="63"/>
+      <c r="D36" s="60"/>
+      <c r="E36" s="61"/>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="30" t="s">
@@ -7839,10 +7962,10 @@
       <c r="C37" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D37" s="62" t="s">
+      <c r="D37" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="E37" s="63"/>
+      <c r="E37" s="61"/>
     </row>
     <row r="38" ht="45" spans="2:5">
       <c r="B38" s="30" t="s">
@@ -7851,61 +7974,61 @@
       <c r="C38" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="D38" s="62"/>
-      <c r="E38" s="73" t="s">
+      <c r="D38" s="60"/>
+      <c r="E38" s="71" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="39" ht="135" spans="2:5">
-      <c r="B39" s="64" t="s">
+      <c r="B39" s="62" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="64"/>
-      <c r="D39" s="64" t="s">
+      <c r="C39" s="62"/>
+      <c r="D39" s="62" t="s">
         <v>130</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="E39" s="26" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="40" ht="135" spans="2:5">
-      <c r="B40" s="64" t="s">
+      <c r="B40" s="62" t="s">
         <v>132</v>
       </c>
-      <c r="C40" s="64"/>
-      <c r="D40" s="64" t="s">
+      <c r="C40" s="62"/>
+      <c r="D40" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="26" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="41" spans="2:5">
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="22" t="s">
         <v>134</v>
       </c>
       <c r="C41" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E41" s="25"/>
+      <c r="E41" s="26"/>
     </row>
     <row r="42" spans="2:5">
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="C42" s="26" t="s">
+      <c r="C42" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="E42" s="25"/>
+      <c r="E42" s="26"/>
     </row>
     <row r="43" spans="2:5">
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="22" t="s">
         <v>138</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="E43" s="25"/>
+      <c r="E43" s="26"/>
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="14" t="s">
@@ -7914,10 +8037,10 @@
       <c r="C44" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="E44" s="25"/>
+      <c r="E44" s="26"/>
     </row>
     <row r="45" ht="195" spans="2:5">
-      <c r="B45" s="21" t="s">
+      <c r="B45" s="22" t="s">
         <v>141</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -7926,24 +8049,24 @@
       <c r="D45" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="E45" s="25"/>
+      <c r="E45" s="26"/>
     </row>
     <row r="46" ht="195" spans="2:5">
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="22" t="s">
         <v>144</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="D46" s="59" t="s">
+      <c r="D46" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="E46" s="49" t="s">
+      <c r="E46" s="48" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="47" ht="195" spans="2:5">
-      <c r="B47" s="21" t="s">
+      <c r="B47" s="22" t="s">
         <v>148</v>
       </c>
       <c r="C47" s="14" t="s">
@@ -7952,7 +8075,7 @@
       <c r="D47" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E47" s="25"/>
+      <c r="E47" s="26"/>
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="14" t="s">
@@ -7961,16 +8084,16 @@
       <c r="C48" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E48" s="25"/>
+      <c r="E48" s="26"/>
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="C49" s="26" t="s">
+      <c r="C49" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="E49" s="25"/>
+      <c r="E49" s="26"/>
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="14" t="s">
@@ -7979,7 +8102,7 @@
       <c r="C50" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="E50" s="25"/>
+      <c r="E50" s="26"/>
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="14" t="s">
@@ -7988,7 +8111,7 @@
       <c r="C51" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="E51" s="25"/>
+      <c r="E51" s="26"/>
     </row>
     <row r="52" ht="150" spans="2:5">
       <c r="B52" s="14" t="s">
@@ -8008,10 +8131,10 @@
       <c r="B53" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="C53" s="26" t="s">
+      <c r="C53" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="E53" s="25"/>
+      <c r="E53" s="26"/>
     </row>
     <row r="54" spans="2:5">
       <c r="B54" s="14" t="s">
@@ -8020,16 +8143,16 @@
       <c r="C54" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="25"/>
+      <c r="E54" s="26"/>
     </row>
     <row r="55" spans="2:5">
       <c r="B55" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="C55" s="26" t="s">
+      <c r="C55" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="E55" s="25"/>
+      <c r="E55" s="26"/>
     </row>
     <row r="56" spans="2:5">
       <c r="B56" s="14" t="s">
@@ -8038,7 +8161,7 @@
       <c r="C56" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="E56" s="25"/>
+      <c r="E56" s="26"/>
     </row>
     <row r="57" spans="2:5">
       <c r="B57" s="14" t="s">
@@ -8047,28 +8170,28 @@
       <c r="C57" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="E57" s="25"/>
+      <c r="E57" s="26"/>
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="C58" s="26" t="s">
+      <c r="C58" s="27" t="s">
         <v>170</v>
       </c>
-      <c r="E58" s="25"/>
+      <c r="E58" s="26"/>
     </row>
     <row r="59" ht="180" spans="2:5">
       <c r="B59" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="C59" s="26" t="s">
+      <c r="C59" s="27" t="s">
         <v>172</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="E59" s="25"/>
+      <c r="E59" s="26"/>
     </row>
     <row r="60" ht="255" spans="2:5">
       <c r="B60" s="14" t="s">
@@ -8080,7 +8203,7 @@
       <c r="D60" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="E60" s="25" t="s">
+      <c r="E60" s="26" t="s">
         <v>177</v>
       </c>
     </row>
@@ -8091,23 +8214,23 @@
       <c r="C61" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="D61" s="65" t="s">
+      <c r="D61" s="63" t="s">
         <v>180</v>
       </c>
-      <c r="E61" s="25"/>
+      <c r="E61" s="26"/>
     </row>
     <row r="62" ht="42.95" customHeight="1" spans="2:5">
       <c r="B62" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="C62" s="61" t="s">
+      <c r="C62" s="59" t="s">
         <v>182</v>
       </c>
-      <c r="D62" s="65"/>
-      <c r="E62" s="25"/>
+      <c r="D62" s="63"/>
+      <c r="E62" s="26"/>
     </row>
     <row r="65" spans="3:3">
-      <c r="C65" s="61"/>
+      <c r="C65" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -8142,32 +8265,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" ht="46" customHeight="1" spans="1:5">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="53" t="s">
         <v>183</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="1:5">
       <c r="B3" s="14" t="s">
@@ -8176,40 +8299,40 @@
       <c r="C3" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="26"/>
     </row>
     <row r="4" ht="90" spans="1:5">
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="54" t="s">
         <v>185</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>26</v>
       </c>
       <c r="C5" t="s">
         <v>187</v>
       </c>
-      <c r="E5" s="25"/>
+      <c r="E5" s="26"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="21" t="s">
         <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>188</v>
       </c>
-      <c r="E6" s="25"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" ht="45" spans="1:5">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C7" t="s">
@@ -8218,18 +8341,18 @@
       <c r="D7" t="s">
         <v>191</v>
       </c>
-      <c r="E7" s="56" t="s">
+      <c r="E7" s="54" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="8" ht="135" spans="1:5">
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="55" t="s">
         <v>193</v>
       </c>
       <c r="C8" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="D8" s="58" t="s">
+      <c r="D8" s="56" t="s">
         <v>195</v>
       </c>
       <c r="E8" s="9" t="s">
@@ -8237,43 +8360,43 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="55" t="s">
         <v>197</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>198</v>
       </c>
       <c r="D9" s="29"/>
-      <c r="E9" s="25"/>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="55" t="s">
         <v>199</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>200</v>
       </c>
       <c r="D10" s="29"/>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="26" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="11" ht="225" spans="1:5">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="21" t="s">
         <v>202</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="57" t="s">
         <v>204</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="26" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>205</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -8284,7 +8407,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>207</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -8295,7 +8418,7 @@
       </c>
     </row>
     <row r="14" ht="30" spans="1:5">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="21" t="s">
         <v>209</v>
       </c>
       <c r="C14" t="s">
@@ -8304,12 +8427,12 @@
       <c r="D14" t="s">
         <v>211</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="26" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="15" ht="135" spans="1:5">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>213</v>
       </c>
       <c r="C15" s="30" t="s">
@@ -8318,12 +8441,12 @@
       <c r="D15" s="30" t="s">
         <v>215</v>
       </c>
-      <c r="E15" s="56" t="s">
+      <c r="E15" s="54" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="16" ht="45" spans="1:5">
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="21" t="s">
         <v>217</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -8332,25 +8455,25 @@
       <c r="D16" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" ht="60" spans="2:5">
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="55" t="s">
         <v>220</v>
       </c>
-      <c r="C17" s="60" t="s">
+      <c r="C17" s="58" t="s">
         <v>221</v>
       </c>
       <c r="D17" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="E17" s="25"/>
+      <c r="E17" s="26"/>
     </row>
     <row r="18" ht="60" spans="2:5">
-      <c r="B18" s="60" t="s">
+      <c r="B18" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="58" t="s">
         <v>224</v>
       </c>
       <c r="D18" s="5" t="s">
@@ -8396,7 +8519,7 @@
       <c r="D21" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="E21" s="25"/>
+      <c r="E21" s="26"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="14" t="s">
@@ -8406,7 +8529,7 @@
         <v>232</v>
       </c>
       <c r="D22" s="14"/>
-      <c r="E22" s="25"/>
+      <c r="E22" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8434,27 +8557,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="25"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="3" spans="1:5">
       <c r="B3" s="14" t="s">
@@ -8463,44 +8586,44 @@
       <c r="C3" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="26"/>
     </row>
     <row r="4" ht="75" spans="1:5">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="48" t="s">
         <v>234</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="20"/>
+      <c r="B5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>52</v>
       </c>
       <c r="D5" s="14"/>
-      <c r="E5" s="25"/>
+      <c r="E5" s="26"/>
     </row>
     <row r="6" ht="30" spans="1:5">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>236</v>
       </c>
       <c r="D6" s="14"/>
-      <c r="E6" s="25"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C7" s="14"/>
@@ -8512,43 +8635,43 @@
       </c>
     </row>
     <row r="8" ht="75" spans="1:5">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="52" t="s">
         <v>239</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="E8" s="74" t="s">
+      <c r="E8" s="72" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="C9" s="54" t="s">
+      <c r="C9" s="52" t="s">
         <v>243</v>
       </c>
       <c r="D9" s="14"/>
-      <c r="E9" s="25"/>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" ht="75" spans="1:5">
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="52" t="s">
         <v>245</v>
       </c>
       <c r="D10" s="14"/>
-      <c r="E10" s="74" t="s">
+      <c r="E10" s="72" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="11" ht="120" spans="1:5">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="21" t="s">
         <v>247</v>
       </c>
       <c r="C11" s="7" t="s">
@@ -8557,26 +8680,26 @@
       <c r="D11" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="E11" s="49" t="s">
+      <c r="E11" s="48" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="12" ht="60" spans="1:5">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="E12" s="51" t="s">
+      <c r="E12" s="15" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>253</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="E13" s="25"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:5">
       <c r="B14" t="s">
@@ -8585,10 +8708,10 @@
       <c r="C14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" ht="75" spans="1:5">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>257</v>
       </c>
       <c r="C15" t="s">
@@ -8597,16 +8720,16 @@
       <c r="D15" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="26"/>
     </row>
     <row r="16" ht="30" spans="1:5">
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="21" t="s">
         <v>260</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" ht="60" spans="2:5">
       <c r="B17" t="s">
@@ -8618,7 +8741,7 @@
       <c r="D17" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="E17" s="25"/>
+      <c r="E17" s="26"/>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" t="s">
@@ -8627,7 +8750,7 @@
       <c r="C18" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="E18" s="25"/>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" ht="30" spans="2:5">
       <c r="B19" t="s">
@@ -8639,7 +8762,7 @@
       <c r="D19" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="26" t="s">
         <v>270</v>
       </c>
     </row>
@@ -8651,7 +8774,7 @@
         <v>272</v>
       </c>
       <c r="D20" s="14"/>
-      <c r="E20" s="25" t="s">
+      <c r="E20" s="26" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8663,7 +8786,7 @@
         <v>275</v>
       </c>
       <c r="D21" s="14"/>
-      <c r="E21" s="25" t="s">
+      <c r="E21" s="26" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8673,7 +8796,7 @@
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="25" t="s">
+      <c r="E22" s="26" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8685,7 +8808,7 @@
         <v>278</v>
       </c>
       <c r="D23" s="14"/>
-      <c r="E23" s="25" t="s">
+      <c r="E23" s="26" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8697,7 +8820,7 @@
       <c r="D24" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="E24" s="25"/>
+      <c r="E24" s="26"/>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" t="s">
@@ -8707,7 +8830,7 @@
         <v>282</v>
       </c>
       <c r="D25" s="14"/>
-      <c r="E25" s="25"/>
+      <c r="E25" s="26"/>
     </row>
     <row r="26" ht="60" spans="2:5">
       <c r="B26" t="s">
@@ -8719,7 +8842,7 @@
       <c r="D26" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="E26" s="25" t="s">
+      <c r="E26" s="26" t="s">
         <v>286</v>
       </c>
     </row>
@@ -8731,7 +8854,7 @@
         <v>288</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="25" t="s">
+      <c r="E27" s="26" t="s">
         <v>286</v>
       </c>
     </row>
@@ -8745,7 +8868,7 @@
       <c r="D28" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="E28" s="25"/>
+      <c r="E28" s="26"/>
     </row>
     <row r="29" ht="30" spans="2:5">
       <c r="B29" s="14" t="s">
@@ -8755,7 +8878,7 @@
         <v>290</v>
       </c>
       <c r="D29" s="14"/>
-      <c r="E29" s="25"/>
+      <c r="E29" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8825,7 +8948,7 @@
       <c r="C4" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="37" t="s">
         <v>294</v>
       </c>
       <c r="E4" s="36"/>
@@ -8852,23 +8975,23 @@
       <c r="E6" s="36"/>
     </row>
     <row r="7" ht="30" spans="1:6">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>296</v>
       </c>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40" t="s">
+      <c r="C7" s="39"/>
+      <c r="D7" s="39" t="s">
         <v>297</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="F7" s="41"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" ht="195" spans="1:6">
       <c r="B8" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="41" t="s">
         <v>300</v>
       </c>
       <c r="D8" s="37" t="s">
@@ -8922,13 +9045,13 @@
       <c r="B13" s="33" t="s">
         <v>310</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="41" t="s">
         <v>311</v>
       </c>
       <c r="D13" s="37" t="s">
         <v>312</v>
       </c>
-      <c r="E13" s="43" t="s">
+      <c r="E13" s="42" t="s">
         <v>313</v>
       </c>
     </row>
@@ -8973,25 +9096,25 @@
       <c r="E17" s="36"/>
     </row>
     <row r="18" ht="30" spans="2:6">
-      <c r="B18" s="44" t="s">
+      <c r="B18" s="43" t="s">
         <v>321</v>
       </c>
-      <c r="C18" s="45" t="s">
+      <c r="C18" s="44" t="s">
         <v>322</v>
       </c>
       <c r="D18" s="37" t="s">
         <v>323</v>
       </c>
-      <c r="E18" s="43" t="s">
+      <c r="E18" s="42" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="19" ht="135" spans="2:6">
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="39" t="s">
         <v>325</v>
       </c>
-      <c r="C19" s="46"/>
-      <c r="D19" s="47" t="s">
+      <c r="C19" s="45"/>
+      <c r="D19" s="46" t="s">
         <v>326</v>
       </c>
       <c r="E19" s="36" t="s">
@@ -9002,11 +9125,11 @@
       <c r="B20" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="47" t="s">
         <v>328</v>
       </c>
       <c r="D20" s="37"/>
-      <c r="E20" s="49" t="s">
+      <c r="E20" s="48" t="s">
         <v>102</v>
       </c>
     </row>
@@ -9014,7 +9137,7 @@
       <c r="B21" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="47" t="s">
         <v>329</v>
       </c>
       <c r="D21" s="37" t="s">
@@ -9026,18 +9149,18 @@
       <c r="B22" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="50" t="s">
+      <c r="C22" s="49" t="s">
         <v>331</v>
       </c>
       <c r="D22" s="37"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="52"/>
-    </row>
-    <row r="23" ht="30" spans="2:6">
+      <c r="E22" s="15"/>
+      <c r="F22" s="50"/>
+    </row>
+    <row r="23" spans="2:6">
       <c r="B23" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="53" t="s">
+      <c r="C23" s="51" t="s">
         <v>332</v>
       </c>
       <c r="D23" s="37" t="s">
@@ -9049,7 +9172,7 @@
       <c r="B24" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" s="47" t="s">
         <v>334</v>
       </c>
       <c r="D24" s="37"/>
@@ -9057,11 +9180,11 @@
         <v>335</v>
       </c>
     </row>
-    <row r="25" ht="45" spans="2:6">
+    <row r="25" ht="30" spans="2:6">
       <c r="B25" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="53" t="s">
+      <c r="C25" s="51" t="s">
         <v>336</v>
       </c>
       <c r="D25" s="37"/>
@@ -9071,7 +9194,7 @@
       <c r="B26" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="48" t="s">
+      <c r="C26" s="47" t="s">
         <v>337</v>
       </c>
       <c r="D26" s="37"/>
@@ -9081,7 +9204,7 @@
       <c r="B27" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C27" s="48" t="s">
+      <c r="C27" s="47" t="s">
         <v>338</v>
       </c>
       <c r="D27" s="37"/>
@@ -9091,7 +9214,7 @@
       <c r="B28" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="48" t="s">
+      <c r="C28" s="47" t="s">
         <v>339</v>
       </c>
       <c r="D28" s="37"/>
@@ -9101,7 +9224,7 @@
       <c r="B29" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="48" t="s">
+      <c r="C29" s="47" t="s">
         <v>340</v>
       </c>
       <c r="D29" s="37"/>
@@ -9111,7 +9234,7 @@
       <c r="B30" s="37" t="s">
         <v>178</v>
       </c>
-      <c r="C30" s="48" t="s">
+      <c r="C30" s="47" t="s">
         <v>179</v>
       </c>
       <c r="D30" s="37" t="s">
@@ -9123,7 +9246,7 @@
       <c r="B31" s="37" t="s">
         <v>181</v>
       </c>
-      <c r="C31" s="53" t="s">
+      <c r="C31" s="51" t="s">
         <v>342</v>
       </c>
       <c r="D31" s="37"/>
@@ -9142,11 +9265,11 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="13.2190476190476" customWidth="1"/>
-    <col min="2" max="2" width="27.2761904761905" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="43.7142857142857" customWidth="1"/>
     <col min="4" max="4" width="47.2857142857143" customWidth="1"/>
     <col min="5" max="5" width="80.5714285714286" customWidth="1"/>
@@ -9154,24 +9277,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="14"/>
@@ -9198,7 +9321,7 @@
       <c r="E4" s="14"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="14" t="s">
@@ -9207,7 +9330,7 @@
       <c r="E5" s="14"/>
     </row>
     <row r="6" ht="30" spans="1:5">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
@@ -9216,19 +9339,19 @@
       <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="22" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="23" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="8" ht="74.25" spans="1:5">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>189</v>
       </c>
       <c r="C8" s="14" t="s">
@@ -9312,7 +9435,7 @@
       <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="22" t="s">
         <v>363</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -9321,7 +9444,7 @@
       <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="22" t="s">
         <v>365</v>
       </c>
       <c r="C16" s="14" t="s">
@@ -9381,7 +9504,7 @@
       <c r="C21" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="17" t="s">
         <v>376</v>
       </c>
       <c r="E21" s="9"/>
@@ -9393,7 +9516,7 @@
       <c r="C22" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="D22" s="16"/>
+      <c r="D22" s="17"/>
       <c r="E22" s="31" t="s">
         <v>379</v>
       </c>
@@ -9403,13 +9526,13 @@
         <v>380</v>
       </c>
       <c r="C23" s="2"/>
-      <c r="D23" s="16"/>
+      <c r="D23" s="17"/>
       <c r="E23" s="12" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="24" ht="75" spans="2:5">
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="22" t="s">
         <v>257</v>
       </c>
       <c r="C24" s="13" t="s">
@@ -9421,7 +9544,7 @@
       <c r="E24" s="14"/>
     </row>
     <row r="25" ht="30" spans="2:5">
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="22" t="s">
         <v>260</v>
       </c>
       <c r="C25" s="14" t="s">
@@ -9442,7 +9565,7 @@
       <c r="E26" s="14"/>
     </row>
     <row r="27" ht="30" spans="2:5">
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="22" t="s">
         <v>387</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -9467,48 +9590,80 @@
       </c>
       <c r="E28" s="14"/>
     </row>
-    <row r="29" ht="30" spans="2:5">
-      <c r="B29" s="14" t="s">
+    <row r="29" s="2" customFormat="1" ht="30" spans="2:5">
+      <c r="B29" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="E29" s="14"/>
-    </row>
-    <row r="30" spans="2:5">
-      <c r="B30" s="14" t="s">
+    </row>
+    <row r="30" s="2" customFormat="1" spans="2:5">
+      <c r="B30" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+    </row>
+    <row r="31" s="2" customFormat="1" ht="270" spans="2:5">
+      <c r="B31" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="15" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="32" ht="30" spans="2:5">
+      <c r="B32" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>402</v>
+      </c>
+      <c r="E32" s="14"/>
+    </row>
+    <row r="33" spans="2:5">
+      <c r="B33" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C33" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="E30" s="14"/>
-    </row>
-    <row r="31" ht="78" customHeight="1" spans="2:5">
-      <c r="B31" s="14" t="s">
+      <c r="D33" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="E33" s="14"/>
+    </row>
+    <row r="34" ht="78" customHeight="1" spans="2:5">
+      <c r="B34" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="C31" s="32" t="s">
-        <v>397</v>
-      </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="C34" s="32" t="s">
+        <v>404</v>
+      </c>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="D9:D13"/>
     <mergeCell ref="D21:D23"/>
-    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="D33:D34"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C31" r:id="rId1" display="&quot;http://shinny.org/us/ny/hrsn/Observation/&lt;observationResourceId&gt;&quot;" tooltip="http://shinny.org/us/ny/hrsn/Observation/&lt;observationResourceId"/>
+    <hyperlink ref="C34" r:id="rId1" display="&quot;http://shinny.org/us/ny/hrsn/Observation/&lt;observationResourceId&gt;&quot;" tooltip="http://shinny.org/us/ny/hrsn/Observation/&lt;observationResourceId"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0.393700787401575" bottom="0.393700787401575" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" pageOrder="overThenDown" orientation="portrait"/>
@@ -9534,78 +9689,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" ht="30" spans="1:5">
-      <c r="A2" s="24" t="s">
-        <v>398</v>
-      </c>
-      <c r="E2" s="25"/>
+      <c r="A2" s="25" t="s">
+        <v>405</v>
+      </c>
+      <c r="E2" s="26"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="19"/>
+      <c r="A3" s="20"/>
       <c r="B3" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="26"/>
     </row>
     <row r="4" ht="90" spans="1:5">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="26" t="s">
-        <v>399</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>400</v>
-      </c>
-      <c r="E4" s="25"/>
+      <c r="C4" s="27" t="s">
+        <v>406</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>407</v>
+      </c>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="20"/>
+      <c r="B5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>52</v>
       </c>
       <c r="D5" s="14"/>
-      <c r="E5" s="25"/>
+      <c r="E5" s="26"/>
     </row>
     <row r="6" ht="30" spans="1:5">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D6" s="14"/>
-      <c r="E6" s="25"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" ht="74.25" spans="1:5">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C7" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="D7" t="s">
         <v>349</v>
@@ -9615,46 +9770,46 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="21" t="s">
         <v>360</v>
       </c>
       <c r="C8" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="D8" s="14"/>
-      <c r="E8" s="25"/>
+      <c r="E8" s="26"/>
     </row>
     <row r="9" ht="42.95" customHeight="1" spans="1:5">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>363</v>
       </c>
       <c r="C9" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>405</v>
-      </c>
-      <c r="E9" s="25"/>
+        <v>412</v>
+      </c>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="21" t="s">
         <v>365</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="27" t="s">
         <v>208</v>
       </c>
       <c r="D10" s="14"/>
-      <c r="E10" s="25"/>
+      <c r="E10" s="26"/>
     </row>
     <row r="11" ht="60.95" customHeight="1" spans="1:5">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="21" t="s">
         <v>366</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="D11" s="14"/>
-      <c r="E11" s="25"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12" ht="30" spans="1:5">
       <c r="B12" s="14" t="s">
@@ -9664,63 +9819,63 @@
         <v>378</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>407</v>
-      </c>
-      <c r="E12" s="25"/>
+        <v>414</v>
+      </c>
+      <c r="E12" s="26"/>
     </row>
     <row r="13" ht="30" spans="1:5">
       <c r="B13" s="14" t="s">
         <v>372</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="D13" s="14"/>
-      <c r="E13" s="25"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" ht="78" customHeight="1" spans="1:5">
       <c r="B14" s="14" t="s">
         <v>373</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="D14" s="14"/>
-      <c r="E14" s="25"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" ht="45" spans="1:5">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>257</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>382</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>410</v>
-      </c>
-      <c r="E15" s="25"/>
+        <v>417</v>
+      </c>
+      <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="21" t="s">
         <v>260</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" ht="30" spans="2:5">
       <c r="B17" t="s">
         <v>387</v>
       </c>
       <c r="C17" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="D17" t="s">
         <v>389</v>
       </c>
-      <c r="E17" s="25" t="s">
-        <v>412</v>
+      <c r="E17" s="26" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="2:5">
@@ -9731,19 +9886,19 @@
         <v>179</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>413</v>
-      </c>
-      <c r="E18" s="25"/>
+        <v>420</v>
+      </c>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="14" t="s">
         <v>181</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="D19" s="14"/>
-      <c r="E19" s="25"/>
+      <c r="E19" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -9771,24 +9926,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>47</v>
       </c>
     </row>
@@ -9797,24 +9952,24 @@
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="D4" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="20"/>
+      <c r="B5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C5" s="14" t="s">
@@ -9824,53 +9979,53 @@
       <c r="E5" s="14"/>
     </row>
     <row r="6" ht="45" spans="1:5">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="D7" t="s">
-        <v>419</v>
-      </c>
-      <c r="E7" s="22"/>
+        <v>426</v>
+      </c>
+      <c r="E7" s="23"/>
     </row>
     <row r="8" ht="165" spans="1:5">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="21" t="s">
         <v>360</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="E8" s="23"/>
+      <c r="E8" s="24"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>363</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="21" t="s">
         <v>365</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -9878,22 +10033,22 @@
         <v>366</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" ht="90" spans="1:5">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>257</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="13" ht="45" spans="1:5">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>260</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -9901,33 +10056,33 @@
       </c>
     </row>
     <row r="14" ht="75" spans="1:5">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="21" t="s">
         <v>384</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>385</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
     </row>
     <row r="15" ht="90" spans="1:5">
       <c r="B15" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="2:4">
@@ -9938,7 +10093,7 @@
         <v>179</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
     </row>
     <row r="18" ht="30" spans="2:4">
@@ -9946,7 +10101,7 @@
         <v>181</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="D18" s="14"/>
     </row>

</xml_diff>